<commit_message>
Update Excel file with anonymised station names
</commit_message>
<xml_diff>
--- a/Retail_Sales_(2024_2025).xlsx
+++ b/Retail_Sales_(2024_2025).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rainoilng-my.sharepoint.com/personal/susan_aigbobhiose_rainoil_com/Documents/Documents/PERSONAL/MBA/YEAR 2/1ST SEMESTER/Data Analytics II/Examination Submission/Exam 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{166112F1-2EBE-4316-8DA0-3D7C5F6718B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD8F5553-876A-4D6D-BF83-BA9696ECEA7D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{24102B43-EB72-4ABC-A4D4-9A62C018D91A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="1008" windowWidth="23256" windowHeight="12456" xr2:uid="{F50D7969-0A5C-4FB3-A32D-D05C2544FBD9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12300" xr2:uid="{F50D7969-0A5C-4FB3-A32D-D05C2544FBD9}"/>
   </bookViews>
   <sheets>
     <sheet name="2024 MOM Station Sale" sheetId="3" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="915" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="915" uniqueCount="430">
   <si>
     <t xml:space="preserve">RETAIL SALES SUMMARY ANALYSIS REPORT - </t>
   </si>
@@ -800,6 +800,537 @@
   <si>
     <t>Area</t>
   </si>
+  <si>
+    <t xml:space="preserve"> Border Road Ikom</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Apo Abuja</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Anwai Road Asaba</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Expressway Asaba</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Highway Calabar</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Nnebisi Road Asaba</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Goldie Road Calabar</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ogoja Road Ikom</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Odukpani</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Uyo Aka Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Makurdi</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Maiduguri</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Uyo Idoro Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Uyo - Abak Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Abakaliki - Azuiyiokwu </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Abakaliki - Mile 50 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Aba - Abayi-Osisioma</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Abijo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Abraka</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> FCT - Gwarimpa </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> FCT - Karmo </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ado-Ekiti - Ikere Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Agbarho - Ohrerhe </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Agbarho - Ewherhe </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Agbor - Asaba Road  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Agbor - Abraka Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Agbor - Alero Road  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Agbor - Owa-Ekei  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Anwai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Asaba - Asaba/Benin Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Asaba - Okpanam Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Auchi - Igara Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Awka - 279 Zik Avenue </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Awka - Regina Caeli Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Awka - 55 Zik Avenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Awkuzu </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ayobo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Kaduna - Barnawa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Benin - Benin/Agbor Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Benin - Benin/Auchi Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Bonsac</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Portharcourt - Borokiri</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Bukuru Jos</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Kaduna - Chikun</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Portharcourt - Choba</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Udu - Steel Town  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Udu - Udu Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> FCT - Dutse Alhaji</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ebrumede</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Warri - Effurun GRA</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Idunmwungha - Egba Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Benin - Ekenwan</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Eket</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ekpoma - Market Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Enugu - Abakpa Nike </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ezenei</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Gboko</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Gombe - Akko</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Gombe - Barunde</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ibafo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ibusa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Igbodo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Portharcourt - Igwuruta</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ikom - Four Corners </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ikom - Calabar Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ilorin - Majeasurawa </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ilorin - Ajase-Ipo Road  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ilorin - Asa Dam Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ilorin - Sobi Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ilorin - Airport Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ipaja</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Portharcourt - Isiokpo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Issele-Uku</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Jarret</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Jeddo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Jesse</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> FCT - Kado</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Kaduna - Kachia Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Kano - Ring Road  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Kano - Danbazo Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Keffi</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Kujama</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Kwale - Umusadege Road  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Kwale - Ogwashi-Ukwu Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Lafia</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Lekki Scheme 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Lokoja</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Benin - Lucky Way</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> FCT - Lugbe</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Makurdi - Atom Kpera </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Minna</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> FCT - New Nyanya</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Nnebisi - 295 Nnebisi Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Nnebisi - 274 Nnebisi Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Nnewi - Oba-Nnewi Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Obiaruku - Novena</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Nsukka</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Obiaruku - Sapele- Agbor New Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Oghara - Ajagbodudu </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Oghara - Otorho Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ogidi - Old Enugu-Onitsha Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ogidi - Ugwu-Nwasike </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ogunnu</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ogwashi-Ukwu - Agidiahen Quarters</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ojodu</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Oke Aro</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Okoh</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Okota</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Okpanam</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Oleh</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Oniru</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Onitsha - 124 Awka Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Onitsha - Modebe </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Oshodi</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Osubi</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Otukpo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Owerri - Orlu Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ozoro - Kwale/ Ozoro Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ozoro - Hospital Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ozoro - Owhelogbo </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Sakponba - Upper Sakponba </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Sakponba - Sakponba Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Saniko</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Sapele - Sapele-Warri Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Sapele - Adeola Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Sapele - Abeke Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Benin - Second East Circular</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Portharcourt - Station Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Asaba - Summit Junction</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ugboko</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ughelli - Amekpa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ughelli - Afiesere </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ughelli - Ekuigbo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ughelli - Iwhrekpokpor </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Benin - Upper Mission</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Benin - Upper Siluko</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Uyo - Atiku Abubakar way</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Warri - PTI Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Warri - Ugbolokposo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Warri - NPA Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Warri - Efurrun/Sapele Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Warri - Anerhen Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Yenagoa - Isaac Boro Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Yenagoa - Edepie </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Yola</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Zaki Biam</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Okwe</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ubiaja</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ibadan - Adegbayi</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Benin By-pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Kwale - Utagba Ogbe </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Umunze</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Nkpor</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Umuahia</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Awada-Obosi</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Agbor - 119 Old Asaba Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Agbor - Owa Ekei/Alero Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Jalingo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Enugu - Nkpokiti</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Koka Junction</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Oleh Ogbemudia Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Auchi - Agenobode</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Anwai Ibori Golf Club</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ogwashi-Ukwu - Poly Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> DSC Otokutu</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Oghara - Otefe</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Idumebo - Irrua</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Eku Town</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Agbor - Alihamie</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Orerokpo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Sagamu</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Yenagoa Opolo-Epie</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Nnewi - Otolo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Okpanam - City Gate</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Irrua - Teaching Hospital</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Udu - Udu Bridge Layout</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Umunede</t>
+  </si>
 </sst>
 </file>
 
@@ -1471,19 +2002,19 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1492,7 +2023,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2029,83 +2560,83 @@
       <c r="F3" s="62"/>
       <c r="G3" s="62"/>
       <c r="H3" s="62"/>
-      <c r="I3" s="56" t="s">
+      <c r="I3" s="57" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="57"/>
+      <c r="J3" s="58"/>
       <c r="K3" s="59"/>
       <c r="L3" s="59"/>
-      <c r="M3" s="58"/>
-      <c r="N3" s="56" t="s">
+      <c r="M3" s="60"/>
+      <c r="N3" s="57" t="s">
         <v>6</v>
       </c>
-      <c r="O3" s="57"/>
+      <c r="O3" s="58"/>
       <c r="P3" s="59"/>
       <c r="Q3" s="59"/>
-      <c r="R3" s="58"/>
-      <c r="S3" s="56" t="s">
+      <c r="R3" s="60"/>
+      <c r="S3" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="T3" s="57"/>
+      <c r="T3" s="58"/>
       <c r="U3" s="59"/>
       <c r="V3" s="59"/>
-      <c r="W3" s="58"/>
-      <c r="X3" s="56" t="s">
+      <c r="W3" s="60"/>
+      <c r="X3" s="57" t="s">
         <v>8</v>
       </c>
-      <c r="Y3" s="57"/>
+      <c r="Y3" s="58"/>
       <c r="Z3" s="59"/>
       <c r="AA3" s="59"/>
-      <c r="AB3" s="58"/>
-      <c r="AC3" s="56" t="s">
+      <c r="AB3" s="60"/>
+      <c r="AC3" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="AD3" s="57"/>
+      <c r="AD3" s="58"/>
       <c r="AE3" s="59"/>
       <c r="AF3" s="59"/>
-      <c r="AG3" s="58"/>
-      <c r="AH3" s="56" t="s">
+      <c r="AG3" s="60"/>
+      <c r="AH3" s="57" t="s">
         <v>10</v>
       </c>
-      <c r="AI3" s="57"/>
+      <c r="AI3" s="58"/>
       <c r="AJ3" s="59"/>
       <c r="AK3" s="59"/>
-      <c r="AL3" s="58"/>
-      <c r="AM3" s="56" t="s">
+      <c r="AL3" s="60"/>
+      <c r="AM3" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="AN3" s="57"/>
+      <c r="AN3" s="58"/>
       <c r="AO3" s="59"/>
       <c r="AP3" s="59"/>
-      <c r="AQ3" s="58"/>
-      <c r="AR3" s="56" t="s">
+      <c r="AQ3" s="60"/>
+      <c r="AR3" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="AS3" s="57"/>
+      <c r="AS3" s="58"/>
       <c r="AT3" s="59"/>
       <c r="AU3" s="59"/>
-      <c r="AV3" s="58"/>
-      <c r="AW3" s="56" t="s">
+      <c r="AV3" s="60"/>
+      <c r="AW3" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="AX3" s="57"/>
+      <c r="AX3" s="58"/>
       <c r="AY3" s="59"/>
       <c r="AZ3" s="59"/>
-      <c r="BA3" s="58"/>
-      <c r="BB3" s="56" t="s">
+      <c r="BA3" s="60"/>
+      <c r="BB3" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="BC3" s="57"/>
+      <c r="BC3" s="58"/>
       <c r="BD3" s="59"/>
       <c r="BE3" s="59"/>
-      <c r="BF3" s="58"/>
-      <c r="BG3" s="56" t="s">
+      <c r="BF3" s="60"/>
+      <c r="BG3" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="BH3" s="57"/>
+      <c r="BH3" s="58"/>
       <c r="BI3" s="59"/>
       <c r="BJ3" s="59"/>
-      <c r="BK3" s="58"/>
+      <c r="BK3" s="60"/>
     </row>
     <row r="4" spans="1:63" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="6"/>
@@ -2300,7 +2831,7 @@
         <v>231</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>21</v>
+        <v>266</v>
       </c>
       <c r="D5" s="17">
         <v>270296</v>
@@ -2491,7 +3022,7 @@
         <v>232</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>22</v>
+        <v>267</v>
       </c>
       <c r="D6" s="17">
         <v>152539</v>
@@ -2682,7 +3213,7 @@
         <v>232</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>23</v>
+        <v>268</v>
       </c>
       <c r="D7" s="17">
         <v>233337</v>
@@ -2873,7 +3404,7 @@
         <v>232</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>24</v>
+        <v>269</v>
       </c>
       <c r="D8" s="17">
         <v>247810</v>
@@ -3064,7 +3595,7 @@
         <v>233</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>25</v>
+        <v>270</v>
       </c>
       <c r="D9" s="17">
         <v>288364</v>
@@ -3255,7 +3786,7 @@
         <v>234</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>26</v>
+        <v>271</v>
       </c>
       <c r="D10" s="17">
         <v>253426</v>
@@ -3446,7 +3977,7 @@
         <v>235</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>27</v>
+        <v>272</v>
       </c>
       <c r="D11" s="17">
         <v>549970</v>
@@ -3637,7 +4168,7 @@
         <v>235</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>28</v>
+        <v>273</v>
       </c>
       <c r="D12" s="17">
         <v>296019</v>
@@ -3828,7 +4359,7 @@
         <v>236</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>29</v>
+        <v>274</v>
       </c>
       <c r="D13" s="17">
         <v>158064</v>
@@ -4019,7 +4550,7 @@
         <v>237</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>30</v>
+        <v>275</v>
       </c>
       <c r="D14" s="17">
         <v>282728</v>
@@ -4210,7 +4741,7 @@
         <v>237</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>31</v>
+        <v>276</v>
       </c>
       <c r="D15" s="17">
         <v>212457</v>
@@ -4401,7 +4932,7 @@
         <v>234</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>32</v>
+        <v>277</v>
       </c>
       <c r="D16" s="17">
         <v>396944</v>
@@ -4592,7 +5123,7 @@
         <v>234</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>33</v>
+        <v>278</v>
       </c>
       <c r="D17" s="17">
         <v>269229</v>
@@ -4783,7 +5314,7 @@
         <v>234</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>34</v>
+        <v>279</v>
       </c>
       <c r="D18" s="17">
         <v>242418</v>
@@ -4974,7 +5505,7 @@
         <v>234</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>35</v>
+        <v>280</v>
       </c>
       <c r="D19" s="17">
         <v>418462</v>
@@ -5165,7 +5696,7 @@
         <v>238</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>36</v>
+        <v>281</v>
       </c>
       <c r="D20" s="17">
         <v>256295</v>
@@ -5356,7 +5887,7 @@
         <v>238</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>37</v>
+        <v>282</v>
       </c>
       <c r="D21" s="17">
         <v>473835</v>
@@ -5547,7 +6078,7 @@
         <v>238</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>38</v>
+        <v>283</v>
       </c>
       <c r="D22" s="17">
         <v>426926</v>
@@ -5738,7 +6269,7 @@
         <v>239</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>39</v>
+        <v>284</v>
       </c>
       <c r="D23" s="17">
         <v>274516</v>
@@ -5929,7 +6460,7 @@
         <v>240</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>40</v>
+        <v>285</v>
       </c>
       <c r="D24" s="17">
         <v>250367</v>
@@ -6120,7 +6651,7 @@
         <v>240</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>41</v>
+        <v>286</v>
       </c>
       <c r="D25" s="17">
         <v>409419</v>
@@ -6311,7 +6842,7 @@
         <v>240</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>42</v>
+        <v>287</v>
       </c>
       <c r="D26" s="17">
         <v>278534</v>
@@ -6502,7 +7033,7 @@
         <v>240</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>43</v>
+        <v>288</v>
       </c>
       <c r="D27" s="17">
         <v>351463</v>
@@ -6693,7 +7224,7 @@
         <v>233</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>44</v>
+        <v>289</v>
       </c>
       <c r="D28" s="17">
         <v>223703</v>
@@ -6884,7 +7415,7 @@
         <v>241</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>45</v>
+        <v>290</v>
       </c>
       <c r="D29" s="17">
         <v>240766</v>
@@ -7075,7 +7606,7 @@
         <v>242</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>46</v>
+        <v>291</v>
       </c>
       <c r="D30" s="17">
         <v>247130</v>
@@ -7266,7 +7797,7 @@
         <v>242</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>47</v>
+        <v>292</v>
       </c>
       <c r="D31" s="17">
         <v>364443</v>
@@ -7457,7 +7988,7 @@
         <v>243</v>
       </c>
       <c r="C32" s="20" t="s">
-        <v>48</v>
+        <v>293</v>
       </c>
       <c r="D32" s="17">
         <v>333454</v>
@@ -7648,7 +8179,7 @@
         <v>231</v>
       </c>
       <c r="C33" s="20" t="s">
-        <v>49</v>
+        <v>253</v>
       </c>
       <c r="D33" s="17">
         <v>323785</v>
@@ -7839,7 +8370,7 @@
         <v>231</v>
       </c>
       <c r="C34" s="20" t="s">
-        <v>50</v>
+        <v>294</v>
       </c>
       <c r="D34" s="17">
         <v>255339</v>
@@ -8030,7 +8561,7 @@
         <v>244</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>51</v>
+        <v>295</v>
       </c>
       <c r="D35" s="17">
         <v>247146</v>
@@ -8221,7 +8752,7 @@
         <v>241</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>52</v>
+        <v>296</v>
       </c>
       <c r="D36" s="17">
         <v>177800</v>
@@ -8412,7 +8943,7 @@
         <v>231</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>53</v>
+        <v>297</v>
       </c>
       <c r="D37" s="17">
         <v>286101</v>
@@ -8603,7 +9134,7 @@
         <v>237</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>54</v>
+        <v>298</v>
       </c>
       <c r="D38" s="17">
         <v>124500</v>
@@ -8794,7 +9325,7 @@
         <v>237</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>55</v>
+        <v>299</v>
       </c>
       <c r="D39" s="17">
         <v>157337</v>
@@ -8985,7 +9516,7 @@
         <v>235</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>56</v>
+        <v>300</v>
       </c>
       <c r="D40" s="17">
         <v>376412</v>
@@ -9176,7 +9707,7 @@
         <v>237</v>
       </c>
       <c r="C41" s="19" t="s">
-        <v>57</v>
+        <v>301</v>
       </c>
       <c r="D41" s="17">
         <v>256789</v>
@@ -9367,7 +9898,7 @@
         <v>237</v>
       </c>
       <c r="C42" s="19" t="s">
-        <v>58</v>
+        <v>302</v>
       </c>
       <c r="D42" s="17">
         <v>257262</v>
@@ -9558,7 +10089,7 @@
         <v>242</v>
       </c>
       <c r="C43" s="19" t="s">
-        <v>59</v>
+        <v>303</v>
       </c>
       <c r="D43" s="17">
         <v>221854</v>
@@ -9749,7 +10280,7 @@
         <v>242</v>
       </c>
       <c r="C44" s="19" t="s">
-        <v>60</v>
+        <v>304</v>
       </c>
       <c r="D44" s="17">
         <v>209820</v>
@@ -9940,7 +10471,7 @@
         <v>231</v>
       </c>
       <c r="C45" s="19" t="s">
-        <v>61</v>
+        <v>305</v>
       </c>
       <c r="D45" s="17">
         <v>221283</v>
@@ -10131,7 +10662,7 @@
         <v>239</v>
       </c>
       <c r="C46" s="19" t="s">
-        <v>62</v>
+        <v>306</v>
       </c>
       <c r="D46" s="17">
         <v>380542</v>
@@ -10513,7 +11044,7 @@
         <v>232</v>
       </c>
       <c r="C48" s="19" t="s">
-        <v>64</v>
+        <v>307</v>
       </c>
       <c r="D48" s="17">
         <v>37369</v>
@@ -10704,7 +11235,7 @@
         <v>238</v>
       </c>
       <c r="C49" s="19" t="s">
-        <v>65</v>
+        <v>308</v>
       </c>
       <c r="D49" s="17">
         <v>242212</v>
@@ -10895,7 +11426,7 @@
         <v>235</v>
       </c>
       <c r="C50" s="19" t="s">
-        <v>66</v>
+        <v>254</v>
       </c>
       <c r="D50" s="17">
         <v>376994</v>
@@ -11086,7 +11617,7 @@
         <v>238</v>
       </c>
       <c r="C51" s="19" t="s">
-        <v>67</v>
+        <v>255</v>
       </c>
       <c r="D51" s="17">
         <v>172509</v>
@@ -11277,7 +11808,7 @@
         <v>238</v>
       </c>
       <c r="C52" s="19" t="s">
-        <v>68</v>
+        <v>256</v>
       </c>
       <c r="D52" s="17">
         <v>752117</v>
@@ -11468,7 +11999,7 @@
         <v>231</v>
       </c>
       <c r="C53" s="19" t="s">
-        <v>69</v>
+        <v>257</v>
       </c>
       <c r="D53" s="17">
         <v>121641</v>
@@ -11659,7 +12190,7 @@
         <v>238</v>
       </c>
       <c r="C54" s="19" t="s">
-        <v>70</v>
+        <v>258</v>
       </c>
       <c r="D54" s="17">
         <v>195321</v>
@@ -11850,7 +12381,7 @@
         <v>244</v>
       </c>
       <c r="C55" s="19" t="s">
-        <v>71</v>
+        <v>309</v>
       </c>
       <c r="D55" s="17">
         <v>166994</v>
@@ -12041,7 +12572,7 @@
         <v>231</v>
       </c>
       <c r="C56" s="19" t="s">
-        <v>72</v>
+        <v>259</v>
       </c>
       <c r="D56" s="17">
         <v>170435</v>
@@ -12232,7 +12763,7 @@
         <v>244</v>
       </c>
       <c r="C57" s="19" t="s">
-        <v>73</v>
+        <v>310</v>
       </c>
       <c r="D57" s="17">
         <v>77171</v>
@@ -12423,7 +12954,7 @@
         <v>244</v>
       </c>
       <c r="C58" s="19" t="s">
-        <v>74</v>
+        <v>311</v>
       </c>
       <c r="D58" s="17">
         <v>16341</v>
@@ -12614,7 +13145,7 @@
         <v>233</v>
       </c>
       <c r="C59" s="19" t="s">
-        <v>75</v>
+        <v>312</v>
       </c>
       <c r="D59" s="17">
         <v>1201421</v>
@@ -12805,7 +13336,7 @@
         <v>243</v>
       </c>
       <c r="C60" s="19" t="s">
-        <v>76</v>
+        <v>313</v>
       </c>
       <c r="D60" s="17">
         <v>239484</v>
@@ -12996,7 +13527,7 @@
         <v>234</v>
       </c>
       <c r="C61" s="19" t="s">
-        <v>77</v>
+        <v>314</v>
       </c>
       <c r="D61" s="17">
         <v>332044</v>
@@ -13187,7 +13718,7 @@
         <v>231</v>
       </c>
       <c r="C62" s="19" t="s">
-        <v>78</v>
+        <v>315</v>
       </c>
       <c r="D62" s="17">
         <v>140599</v>
@@ -13378,7 +13909,7 @@
         <v>245</v>
       </c>
       <c r="C63" s="19" t="s">
-        <v>79</v>
+        <v>316</v>
       </c>
       <c r="D63" s="17">
         <v>417660</v>
@@ -13569,7 +14100,7 @@
         <v>245</v>
       </c>
       <c r="C64" s="20" t="s">
-        <v>80</v>
+        <v>260</v>
       </c>
       <c r="D64" s="17">
         <v>269441</v>
@@ -13760,7 +14291,7 @@
         <v>245</v>
       </c>
       <c r="C65" s="19" t="s">
-        <v>81</v>
+        <v>317</v>
       </c>
       <c r="D65" s="17">
         <v>499302</v>
@@ -13951,7 +14482,7 @@
         <v>236</v>
       </c>
       <c r="C66" s="19" t="s">
-        <v>82</v>
+        <v>318</v>
       </c>
       <c r="D66" s="17">
         <v>221877</v>
@@ -14142,7 +14673,7 @@
         <v>236</v>
       </c>
       <c r="C67" s="19" t="s">
-        <v>83</v>
+        <v>319</v>
       </c>
       <c r="D67" s="17">
         <v>230674</v>
@@ -14333,7 +14864,7 @@
         <v>236</v>
       </c>
       <c r="C68" s="19" t="s">
-        <v>84</v>
+        <v>320</v>
       </c>
       <c r="D68" s="17">
         <v>216563</v>
@@ -14524,7 +15055,7 @@
         <v>236</v>
       </c>
       <c r="C69" s="19" t="s">
-        <v>85</v>
+        <v>321</v>
       </c>
       <c r="D69" s="17">
         <v>209906</v>
@@ -14715,7 +15246,7 @@
         <v>236</v>
       </c>
       <c r="C70" s="19" t="s">
-        <v>86</v>
+        <v>322</v>
       </c>
       <c r="D70" s="17">
         <v>165855</v>
@@ -14906,7 +15437,7 @@
         <v>233</v>
       </c>
       <c r="C71" s="19" t="s">
-        <v>87</v>
+        <v>323</v>
       </c>
       <c r="D71" s="17">
         <v>537750</v>
@@ -15097,7 +15628,7 @@
         <v>231</v>
       </c>
       <c r="C72" s="19" t="s">
-        <v>88</v>
+        <v>324</v>
       </c>
       <c r="D72" s="17">
         <v>98494</v>
@@ -15288,7 +15819,7 @@
         <v>243</v>
       </c>
       <c r="C73" s="19" t="s">
-        <v>89</v>
+        <v>325</v>
       </c>
       <c r="D73" s="17">
         <v>230607</v>
@@ -15479,7 +16010,7 @@
         <v>238</v>
       </c>
       <c r="C74" s="19" t="s">
-        <v>90</v>
+        <v>326</v>
       </c>
       <c r="D74" s="17">
         <v>104621</v>
@@ -15670,7 +16201,7 @@
         <v>237</v>
       </c>
       <c r="C75" s="19" t="s">
-        <v>91</v>
+        <v>327</v>
       </c>
       <c r="D75" s="17">
         <v>153751</v>
@@ -15861,7 +16392,7 @@
         <v>246</v>
       </c>
       <c r="C76" s="19" t="s">
-        <v>92</v>
+        <v>328</v>
       </c>
       <c r="D76" s="17">
         <v>175569</v>
@@ -16052,7 +16583,7 @@
         <v>235</v>
       </c>
       <c r="C77" s="19" t="s">
-        <v>93</v>
+        <v>329</v>
       </c>
       <c r="D77" s="17">
         <v>300054</v>
@@ -16434,7 +16965,7 @@
         <v>241</v>
       </c>
       <c r="C79" s="19" t="s">
-        <v>95</v>
+        <v>330</v>
       </c>
       <c r="D79" s="17">
         <v>103121</v>
@@ -16625,7 +17156,7 @@
         <v>241</v>
       </c>
       <c r="C80" s="19" t="s">
-        <v>96</v>
+        <v>331</v>
       </c>
       <c r="D80" s="17">
         <v>108712</v>
@@ -16816,7 +17347,7 @@
         <v>241</v>
       </c>
       <c r="C81" s="19" t="s">
-        <v>97</v>
+        <v>332</v>
       </c>
       <c r="D81" s="17">
         <v>112050</v>
@@ -17007,7 +17538,7 @@
         <v>235</v>
       </c>
       <c r="C82" s="19" t="s">
-        <v>98</v>
+        <v>333</v>
       </c>
       <c r="D82" s="17">
         <v>226986</v>
@@ -17198,7 +17729,7 @@
         <v>241</v>
       </c>
       <c r="C83" s="19" t="s">
-        <v>99</v>
+        <v>334</v>
       </c>
       <c r="D83" s="17">
         <v>115002</v>
@@ -17389,7 +17920,7 @@
         <v>243</v>
       </c>
       <c r="C84" s="19" t="s">
-        <v>100</v>
+        <v>335</v>
       </c>
       <c r="D84" s="17">
         <v>291527</v>
@@ -17580,7 +18111,7 @@
         <v>243</v>
       </c>
       <c r="C85" s="19" t="s">
-        <v>101</v>
+        <v>336</v>
       </c>
       <c r="D85" s="17">
         <v>269033</v>
@@ -17771,7 +18302,7 @@
         <v>244</v>
       </c>
       <c r="C86" s="19" t="s">
-        <v>102</v>
+        <v>337</v>
       </c>
       <c r="D86" s="17">
         <v>284585</v>
@@ -17962,7 +18493,7 @@
         <v>233</v>
       </c>
       <c r="C87" s="19" t="s">
-        <v>103</v>
+        <v>338</v>
       </c>
       <c r="D87" s="17">
         <v>271210</v>
@@ -18153,7 +18684,7 @@
         <v>235</v>
       </c>
       <c r="C88" s="19" t="s">
-        <v>104</v>
+        <v>339</v>
       </c>
       <c r="D88" s="17">
         <v>238736</v>
@@ -18344,7 +18875,7 @@
         <v>242</v>
       </c>
       <c r="C89" s="19" t="s">
-        <v>105</v>
+        <v>340</v>
       </c>
       <c r="D89" s="17">
         <v>194081</v>
@@ -18535,7 +19066,7 @@
         <v>235</v>
       </c>
       <c r="C90" s="19" t="s">
-        <v>106</v>
+        <v>341</v>
       </c>
       <c r="D90" s="17">
         <v>179557</v>
@@ -18726,7 +19257,7 @@
         <v>244</v>
       </c>
       <c r="C91" s="20" t="s">
-        <v>107</v>
+        <v>342</v>
       </c>
       <c r="D91" s="17">
         <v>217549</v>
@@ -18917,7 +19448,7 @@
         <v>235</v>
       </c>
       <c r="C92" s="19" t="s">
-        <v>108</v>
+        <v>343</v>
       </c>
       <c r="D92" s="17">
         <v>94558</v>
@@ -19108,7 +19639,7 @@
         <v>235</v>
       </c>
       <c r="C93" s="19" t="s">
-        <v>109</v>
+        <v>344</v>
       </c>
       <c r="D93" s="17">
         <v>74936</v>
@@ -19299,7 +19830,7 @@
         <v>238</v>
       </c>
       <c r="C94" s="20" t="s">
-        <v>110</v>
+        <v>345</v>
       </c>
       <c r="D94" s="17">
         <v>451245</v>
@@ -19490,7 +20021,7 @@
         <v>238</v>
       </c>
       <c r="C95" s="20" t="s">
-        <v>111</v>
+        <v>346</v>
       </c>
       <c r="D95" s="17">
         <v>226484</v>
@@ -19681,7 +20212,7 @@
         <v>240</v>
       </c>
       <c r="C96" s="19" t="s">
-        <v>112</v>
+        <v>347</v>
       </c>
       <c r="D96" s="17">
         <v>275290</v>
@@ -19872,7 +20403,7 @@
         <v>247</v>
       </c>
       <c r="C97" s="19" t="s">
-        <v>113</v>
+        <v>348</v>
       </c>
       <c r="D97" s="17">
         <v>335503</v>
@@ -20063,7 +20594,7 @@
         <v>232</v>
       </c>
       <c r="C98" s="19" t="s">
-        <v>114</v>
+        <v>349</v>
       </c>
       <c r="D98" s="17">
         <v>370323</v>
@@ -20254,7 +20785,7 @@
         <v>247</v>
       </c>
       <c r="C99" s="20" t="s">
-        <v>115</v>
+        <v>350</v>
       </c>
       <c r="D99" s="17">
         <v>227499</v>
@@ -20445,7 +20976,7 @@
         <v>231</v>
       </c>
       <c r="C100" s="20" t="s">
-        <v>116</v>
+        <v>261</v>
       </c>
       <c r="D100" s="17">
         <v>204727</v>
@@ -20636,7 +21167,7 @@
         <v>246</v>
       </c>
       <c r="C101" s="19" t="s">
-        <v>117</v>
+        <v>351</v>
       </c>
       <c r="D101" s="17">
         <v>240338</v>
@@ -20827,7 +21358,7 @@
         <v>246</v>
       </c>
       <c r="C102" s="19" t="s">
-        <v>118</v>
+        <v>352</v>
       </c>
       <c r="D102" s="17">
         <v>344348</v>
@@ -21018,7 +21549,7 @@
         <v>240</v>
       </c>
       <c r="C103" s="19" t="s">
-        <v>119</v>
+        <v>353</v>
       </c>
       <c r="D103" s="17">
         <v>169071</v>
@@ -21209,7 +21740,7 @@
         <v>240</v>
       </c>
       <c r="C104" s="19" t="s">
-        <v>120</v>
+        <v>354</v>
       </c>
       <c r="D104" s="17">
         <v>206323</v>
@@ -21400,7 +21931,7 @@
         <v>237</v>
       </c>
       <c r="C105" s="19" t="s">
-        <v>121</v>
+        <v>355</v>
       </c>
       <c r="D105" s="17">
         <v>254093</v>
@@ -21591,7 +22122,7 @@
         <v>243</v>
       </c>
       <c r="C106" s="19" t="s">
-        <v>122</v>
+        <v>356</v>
       </c>
       <c r="D106" s="17">
         <v>381070</v>
@@ -21782,7 +22313,7 @@
         <v>233</v>
       </c>
       <c r="C107" s="19" t="s">
-        <v>123</v>
+        <v>357</v>
       </c>
       <c r="D107" s="17">
         <v>232379</v>
@@ -21973,7 +22504,7 @@
         <v>233</v>
       </c>
       <c r="C108" s="19" t="s">
-        <v>124</v>
+        <v>358</v>
       </c>
       <c r="D108" s="17">
         <v>202963</v>
@@ -22164,7 +22695,7 @@
         <v>240</v>
       </c>
       <c r="C109" s="19" t="s">
-        <v>125</v>
+        <v>359</v>
       </c>
       <c r="D109" s="17">
         <v>244953</v>
@@ -22355,7 +22886,7 @@
         <v>233</v>
       </c>
       <c r="C110" s="19" t="s">
-        <v>126</v>
+        <v>360</v>
       </c>
       <c r="D110" s="17">
         <v>340283</v>
@@ -22546,7 +23077,7 @@
         <v>243</v>
       </c>
       <c r="C111" s="20" t="s">
-        <v>127</v>
+        <v>361</v>
       </c>
       <c r="D111" s="17">
         <v>257802</v>
@@ -22737,7 +23268,7 @@
         <v>247</v>
       </c>
       <c r="C112" s="19" t="s">
-        <v>128</v>
+        <v>362</v>
       </c>
       <c r="D112" s="17">
         <v>452004</v>
@@ -22928,7 +23459,7 @@
         <v>233</v>
       </c>
       <c r="C113" s="19" t="s">
-        <v>129</v>
+        <v>363</v>
       </c>
       <c r="D113" s="17">
         <v>473858</v>
@@ -23119,7 +23650,7 @@
         <v>240</v>
       </c>
       <c r="C114" s="19" t="s">
-        <v>130</v>
+        <v>364</v>
       </c>
       <c r="D114" s="17">
         <v>355859</v>
@@ -23310,7 +23841,7 @@
         <v>240</v>
       </c>
       <c r="C115" s="19" t="s">
-        <v>131</v>
+        <v>365</v>
       </c>
       <c r="D115" s="17">
         <v>249779</v>
@@ -23501,7 +24032,7 @@
         <v>233</v>
       </c>
       <c r="C116" s="19" t="s">
-        <v>132</v>
+        <v>366</v>
       </c>
       <c r="D116" s="17">
         <v>384676</v>
@@ -23692,7 +24223,7 @@
         <v>237</v>
       </c>
       <c r="C117" s="19" t="s">
-        <v>133</v>
+        <v>367</v>
       </c>
       <c r="D117" s="17">
         <v>308077</v>
@@ -23883,7 +24414,7 @@
         <v>244</v>
       </c>
       <c r="C118" s="19" t="s">
-        <v>134</v>
+        <v>368</v>
       </c>
       <c r="D118" s="17">
         <v>130034</v>
@@ -24074,7 +24605,7 @@
         <v>232</v>
       </c>
       <c r="C119" s="19" t="s">
-        <v>135</v>
+        <v>369</v>
       </c>
       <c r="D119" s="17">
         <v>191059</v>
@@ -24265,7 +24796,7 @@
         <v>247</v>
       </c>
       <c r="C120" s="19" t="s">
-        <v>136</v>
+        <v>370</v>
       </c>
       <c r="D120" s="17">
         <v>285563</v>
@@ -24456,7 +24987,7 @@
         <v>247</v>
       </c>
       <c r="C121" s="19" t="s">
-        <v>137</v>
+        <v>371</v>
       </c>
       <c r="D121" s="17">
         <v>288253</v>
@@ -24647,7 +25178,7 @@
         <v>247</v>
       </c>
       <c r="C122" s="19" t="s">
-        <v>138</v>
+        <v>372</v>
       </c>
       <c r="D122" s="17">
         <v>362377</v>
@@ -24838,7 +25369,7 @@
         <v>242</v>
       </c>
       <c r="C123" s="19" t="s">
-        <v>139</v>
+        <v>373</v>
       </c>
       <c r="D123" s="17">
         <v>289502</v>
@@ -25029,7 +25560,7 @@
         <v>242</v>
       </c>
       <c r="C124" s="19" t="s">
-        <v>140</v>
+        <v>374</v>
       </c>
       <c r="D124" s="17">
         <v>201700</v>
@@ -25220,7 +25751,7 @@
         <v>248</v>
       </c>
       <c r="C125" s="19" t="s">
-        <v>141</v>
+        <v>375</v>
       </c>
       <c r="D125" s="17">
         <v>260880</v>
@@ -25411,7 +25942,7 @@
         <v>246</v>
       </c>
       <c r="C126" s="19" t="s">
-        <v>142</v>
+        <v>376</v>
       </c>
       <c r="D126" s="17">
         <v>245504</v>
@@ -25602,7 +26133,7 @@
         <v>246</v>
       </c>
       <c r="C127" s="19" t="s">
-        <v>143</v>
+        <v>377</v>
       </c>
       <c r="D127" s="17">
         <v>112136</v>
@@ -25793,7 +26324,7 @@
         <v>246</v>
       </c>
       <c r="C128" s="19" t="s">
-        <v>144</v>
+        <v>378</v>
       </c>
       <c r="D128" s="17">
         <v>182765</v>
@@ -25984,7 +26515,7 @@
         <v>242</v>
       </c>
       <c r="C129" s="19" t="s">
-        <v>145</v>
+        <v>379</v>
       </c>
       <c r="D129" s="17">
         <v>179965</v>
@@ -26175,7 +26706,7 @@
         <v>231</v>
       </c>
       <c r="C130" s="19" t="s">
-        <v>146</v>
+        <v>380</v>
       </c>
       <c r="D130" s="17">
         <v>345306</v>
@@ -26366,7 +26897,7 @@
         <v>238</v>
       </c>
       <c r="C131" s="19" t="s">
-        <v>147</v>
+        <v>381</v>
       </c>
       <c r="D131" s="17">
         <v>1415623</v>
@@ -26557,7 +27088,7 @@
         <v>243</v>
       </c>
       <c r="C132" s="19" t="s">
-        <v>148</v>
+        <v>382</v>
       </c>
       <c r="D132" s="17">
         <v>118520</v>
@@ -26748,7 +27279,7 @@
         <v>248</v>
       </c>
       <c r="C133" s="19" t="s">
-        <v>149</v>
+        <v>383</v>
       </c>
       <c r="D133" s="17">
         <v>359766</v>
@@ -26939,7 +27470,7 @@
         <v>248</v>
       </c>
       <c r="C134" s="19" t="s">
-        <v>150</v>
+        <v>384</v>
       </c>
       <c r="D134" s="17">
         <v>252796</v>
@@ -27130,7 +27661,7 @@
         <v>248</v>
       </c>
       <c r="C135" s="19" t="s">
-        <v>151</v>
+        <v>385</v>
       </c>
       <c r="D135" s="17">
         <v>276448</v>
@@ -27321,7 +27852,7 @@
         <v>248</v>
       </c>
       <c r="C136" s="19" t="s">
-        <v>152</v>
+        <v>386</v>
       </c>
       <c r="D136" s="17">
         <v>270894</v>
@@ -27512,7 +28043,7 @@
         <v>242</v>
       </c>
       <c r="C137" s="19" t="s">
-        <v>153</v>
+        <v>387</v>
       </c>
       <c r="D137" s="17">
         <v>313140</v>
@@ -27703,7 +28234,7 @@
         <v>242</v>
       </c>
       <c r="C138" s="19" t="s">
-        <v>154</v>
+        <v>388</v>
       </c>
       <c r="D138" s="17">
         <v>177686</v>
@@ -27894,7 +28425,7 @@
         <v>231</v>
       </c>
       <c r="C139" s="19" t="s">
-        <v>155</v>
+        <v>389</v>
       </c>
       <c r="D139" s="17">
         <v>463904</v>
@@ -28085,7 +28616,7 @@
         <v>237</v>
       </c>
       <c r="C140" s="19" t="s">
-        <v>156</v>
+        <v>390</v>
       </c>
       <c r="D140" s="17">
         <v>120242</v>
@@ -28276,7 +28807,7 @@
         <v>237</v>
       </c>
       <c r="C141" s="19" t="s">
-        <v>157</v>
+        <v>391</v>
       </c>
       <c r="D141" s="17">
         <v>135211</v>
@@ -28467,7 +28998,7 @@
         <v>237</v>
       </c>
       <c r="C142" s="19" t="s">
-        <v>158</v>
+        <v>392</v>
       </c>
       <c r="D142" s="17">
         <v>238484</v>
@@ -28658,7 +29189,7 @@
         <v>237</v>
       </c>
       <c r="C143" s="19" t="s">
-        <v>159</v>
+        <v>393</v>
       </c>
       <c r="D143" s="17">
         <v>114293</v>
@@ -28849,7 +29380,7 @@
         <v>237</v>
       </c>
       <c r="C144" s="19" t="s">
-        <v>160</v>
+        <v>394</v>
       </c>
       <c r="D144" s="17">
         <v>74101</v>
@@ -29040,7 +29571,7 @@
         <v>249</v>
       </c>
       <c r="C145" s="19" t="s">
-        <v>161</v>
+        <v>395</v>
       </c>
       <c r="D145" s="17">
         <v>408049</v>
@@ -29231,7 +29762,7 @@
         <v>249</v>
       </c>
       <c r="C146" s="19" t="s">
-        <v>162</v>
+        <v>396</v>
       </c>
       <c r="D146" s="17">
         <v>385460</v>
@@ -29422,7 +29953,7 @@
         <v>250</v>
       </c>
       <c r="C147" s="19" t="s">
-        <v>163</v>
+        <v>397</v>
       </c>
       <c r="D147" s="17">
         <v>69786</v>
@@ -29613,7 +30144,7 @@
         <v>244</v>
       </c>
       <c r="C148" s="19" t="s">
-        <v>164</v>
+        <v>398</v>
       </c>
       <c r="D148" s="17">
         <v>120113</v>
@@ -29804,7 +30335,7 @@
         <v>243</v>
       </c>
       <c r="C149" s="19" t="s">
-        <v>165</v>
+        <v>399</v>
       </c>
       <c r="D149" s="17">
         <v>218576</v>
@@ -29995,7 +30526,7 @@
         <v>239</v>
       </c>
       <c r="C150" s="19" t="s">
-        <v>166</v>
+        <v>400</v>
       </c>
       <c r="D150" s="17">
         <v>250795</v>
@@ -30186,7 +30717,7 @@
         <v>236</v>
       </c>
       <c r="C151" s="19" t="s">
-        <v>167</v>
+        <v>401</v>
       </c>
       <c r="D151" s="17">
         <v>281863</v>
@@ -30377,7 +30908,7 @@
         <v>242</v>
       </c>
       <c r="C152" s="19" t="s">
-        <v>168</v>
+        <v>402</v>
       </c>
       <c r="D152" s="17">
         <v>452079</v>
@@ -30568,7 +31099,7 @@
         <v>243</v>
       </c>
       <c r="C153" s="19" t="s">
-        <v>169</v>
+        <v>403</v>
       </c>
       <c r="D153" s="17">
         <v>122963</v>
@@ -30759,7 +31290,7 @@
         <v>240</v>
       </c>
       <c r="C154" s="19" t="s">
-        <v>170</v>
+        <v>404</v>
       </c>
       <c r="D154" s="17">
         <v>219770</v>
@@ -30950,7 +31481,7 @@
         <v>240</v>
       </c>
       <c r="C155" s="19" t="s">
-        <v>171</v>
+        <v>405</v>
       </c>
       <c r="D155" s="17">
         <v>146894</v>
@@ -31141,7 +31672,7 @@
         <v>232</v>
       </c>
       <c r="C156" s="19" t="s">
-        <v>172</v>
+        <v>406</v>
       </c>
       <c r="D156" s="17">
         <v>281085</v>
@@ -31332,7 +31863,7 @@
         <v>240</v>
       </c>
       <c r="C157" s="19" t="s">
-        <v>173</v>
+        <v>407</v>
       </c>
       <c r="D157" s="17">
         <v>121637</v>
@@ -31523,7 +32054,7 @@
         <v>234</v>
       </c>
       <c r="C158" s="19" t="s">
-        <v>174</v>
+        <v>408</v>
       </c>
       <c r="D158" s="17">
         <v>396601</v>
@@ -31714,7 +32245,7 @@
         <v>234</v>
       </c>
       <c r="C159" s="19" t="s">
-        <v>175</v>
+        <v>409</v>
       </c>
       <c r="D159" s="17">
         <v>335693</v>
@@ -31905,7 +32436,7 @@
         <v>231</v>
       </c>
       <c r="C160" s="19" t="s">
-        <v>176</v>
+        <v>262</v>
       </c>
       <c r="D160" s="17">
         <v>275507</v>
@@ -32096,7 +32627,7 @@
         <v>250</v>
       </c>
       <c r="C161" s="19" t="s">
-        <v>177</v>
+        <v>410</v>
       </c>
       <c r="D161" s="17">
         <v>248876</v>
@@ -32287,7 +32818,7 @@
         <v>232</v>
       </c>
       <c r="C162" s="19" t="s">
-        <v>178</v>
+        <v>411</v>
       </c>
       <c r="D162" s="17">
         <v>325379</v>
@@ -32478,7 +33009,7 @@
         <v>238</v>
       </c>
       <c r="C163" s="19" t="s">
-        <v>179</v>
+        <v>412</v>
       </c>
       <c r="D163" s="17">
         <v>442136</v>
@@ -32669,7 +33200,7 @@
         <v>247</v>
       </c>
       <c r="C164" s="19" t="s">
-        <v>180</v>
+        <v>413</v>
       </c>
       <c r="D164" s="17">
         <v>187555</v>
@@ -32860,7 +33391,7 @@
         <v>244</v>
       </c>
       <c r="C165" s="19" t="s">
-        <v>181</v>
+        <v>263</v>
       </c>
       <c r="D165" s="17">
         <v>221425</v>
@@ -33051,7 +33582,7 @@
         <v>239</v>
       </c>
       <c r="C166" s="19" t="s">
-        <v>182</v>
+        <v>414</v>
       </c>
       <c r="D166" s="17">
         <v>212518</v>
@@ -33242,7 +33773,7 @@
         <v>238</v>
       </c>
       <c r="C167" s="19" t="s">
-        <v>183</v>
+        <v>415</v>
       </c>
       <c r="D167" s="17">
         <v>251938</v>
@@ -33433,7 +33964,7 @@
         <v>243</v>
       </c>
       <c r="C168" s="19" t="s">
-        <v>184</v>
+        <v>416</v>
       </c>
       <c r="D168" s="17">
         <v>145041</v>
@@ -33624,7 +34155,7 @@
         <v>248</v>
       </c>
       <c r="C169" s="19" t="s">
-        <v>185</v>
+        <v>417</v>
       </c>
       <c r="D169" s="17">
         <v>177367</v>
@@ -33815,7 +34346,7 @@
         <v>246</v>
       </c>
       <c r="C170" s="19" t="s">
-        <v>186</v>
+        <v>418</v>
       </c>
       <c r="D170" s="17">
         <v>190380</v>
@@ -34006,7 +34537,7 @@
         <v>239</v>
       </c>
       <c r="C171" s="19" t="s">
-        <v>187</v>
+        <v>419</v>
       </c>
       <c r="D171" s="17">
         <v>356098</v>
@@ -34197,7 +34728,7 @@
         <v>247</v>
       </c>
       <c r="C172" s="19" t="s">
-        <v>188</v>
+        <v>420</v>
       </c>
       <c r="D172" s="17">
         <v>176255</v>
@@ -34388,7 +34919,7 @@
         <v>250</v>
       </c>
       <c r="C173" s="19" t="s">
-        <v>189</v>
+        <v>264</v>
       </c>
       <c r="D173" s="17">
         <v>0</v>
@@ -34579,7 +35110,7 @@
         <v>234</v>
       </c>
       <c r="C174" s="19" t="s">
-        <v>190</v>
+        <v>421</v>
       </c>
       <c r="D174" s="17">
         <v>0</v>
@@ -34770,7 +35301,7 @@
         <v>237</v>
       </c>
       <c r="C175" s="19" t="s">
-        <v>191</v>
+        <v>422</v>
       </c>
       <c r="D175" s="17">
         <v>0</v>
@@ -34961,7 +35492,7 @@
         <v>231</v>
       </c>
       <c r="C176" s="19" t="s">
-        <v>192</v>
+        <v>265</v>
       </c>
       <c r="D176" s="17">
         <v>0</v>
@@ -35152,7 +35683,7 @@
         <v>233</v>
       </c>
       <c r="C177" s="19" t="s">
-        <v>193</v>
+        <v>423</v>
       </c>
       <c r="D177" s="17">
         <v>0</v>
@@ -35343,7 +35874,7 @@
         <v>249</v>
       </c>
       <c r="C178" s="19" t="s">
-        <v>194</v>
+        <v>424</v>
       </c>
       <c r="D178" s="17">
         <v>0</v>
@@ -35534,7 +36065,7 @@
         <v>251</v>
       </c>
       <c r="C179" s="22" t="s">
-        <v>195</v>
+        <v>425</v>
       </c>
       <c r="D179" s="17">
         <v>0</v>
@@ -35725,7 +36256,7 @@
         <v>243</v>
       </c>
       <c r="C180" s="19" t="s">
-        <v>196</v>
+        <v>426</v>
       </c>
       <c r="D180" s="17">
         <v>0</v>
@@ -35916,7 +36447,7 @@
         <v>239</v>
       </c>
       <c r="C181" s="19" t="s">
-        <v>197</v>
+        <v>427</v>
       </c>
       <c r="D181" s="17">
         <v>0</v>
@@ -36107,7 +36638,7 @@
         <v>237</v>
       </c>
       <c r="C182" s="19" t="s">
-        <v>198</v>
+        <v>428</v>
       </c>
       <c r="D182" s="17">
         <v>0</v>
@@ -36294,11 +36825,11 @@
       <c r="A183" s="18">
         <v>179</v>
       </c>
-      <c r="B183" s="63" t="s">
+      <c r="B183" s="56" t="s">
         <v>234</v>
       </c>
       <c r="C183" s="19" t="s">
-        <v>199</v>
+        <v>429</v>
       </c>
       <c r="D183" s="17">
         <v>0</v>
@@ -37136,87 +37667,87 @@
       <c r="C3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="56" t="s">
+      <c r="D3" s="57" t="s">
         <v>203</v>
       </c>
-      <c r="E3" s="57"/>
-      <c r="F3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="60"/>
       <c r="G3" s="29"/>
       <c r="H3" s="29"/>
-      <c r="I3" s="60" t="s">
+      <c r="I3" s="63" t="s">
         <v>204</v>
       </c>
-      <c r="J3" s="57"/>
-      <c r="K3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="60"/>
       <c r="L3" s="29"/>
       <c r="M3" s="29"/>
-      <c r="N3" s="56" t="s">
+      <c r="N3" s="57" t="s">
         <v>205</v>
       </c>
-      <c r="O3" s="57"/>
-      <c r="P3" s="58"/>
+      <c r="O3" s="58"/>
+      <c r="P3" s="60"/>
       <c r="Q3" s="29"/>
       <c r="R3" s="29"/>
-      <c r="S3" s="56" t="s">
+      <c r="S3" s="57" t="s">
         <v>206</v>
       </c>
-      <c r="T3" s="57"/>
-      <c r="U3" s="58"/>
+      <c r="T3" s="58"/>
+      <c r="U3" s="60"/>
       <c r="V3" s="29"/>
       <c r="W3" s="29"/>
-      <c r="X3" s="56" t="s">
+      <c r="X3" s="57" t="s">
         <v>207</v>
       </c>
-      <c r="Y3" s="57"/>
-      <c r="Z3" s="58"/>
+      <c r="Y3" s="58"/>
+      <c r="Z3" s="60"/>
       <c r="AA3" s="29"/>
       <c r="AB3" s="29"/>
-      <c r="AC3" s="56" t="s">
+      <c r="AC3" s="57" t="s">
         <v>208</v>
       </c>
-      <c r="AD3" s="57"/>
-      <c r="AE3" s="58"/>
+      <c r="AD3" s="58"/>
+      <c r="AE3" s="60"/>
       <c r="AF3" s="29"/>
       <c r="AG3" s="29"/>
-      <c r="AH3" s="56" t="s">
+      <c r="AH3" s="57" t="s">
         <v>209</v>
       </c>
-      <c r="AI3" s="57"/>
-      <c r="AJ3" s="58"/>
+      <c r="AI3" s="58"/>
+      <c r="AJ3" s="60"/>
       <c r="AK3" s="29"/>
       <c r="AL3" s="29"/>
-      <c r="AM3" s="56" t="s">
+      <c r="AM3" s="57" t="s">
         <v>210</v>
       </c>
-      <c r="AN3" s="57"/>
-      <c r="AO3" s="58"/>
+      <c r="AN3" s="58"/>
+      <c r="AO3" s="60"/>
       <c r="AP3" s="29"/>
       <c r="AQ3" s="29"/>
-      <c r="AR3" s="56" t="s">
+      <c r="AR3" s="57" t="s">
         <v>211</v>
       </c>
-      <c r="AS3" s="57"/>
-      <c r="AT3" s="58"/>
+      <c r="AS3" s="58"/>
+      <c r="AT3" s="60"/>
       <c r="AU3" s="29"/>
       <c r="AV3" s="29"/>
-      <c r="AW3" s="56" t="s">
+      <c r="AW3" s="57" t="s">
         <v>212</v>
       </c>
-      <c r="AX3" s="57"/>
-      <c r="AY3" s="58"/>
+      <c r="AX3" s="58"/>
+      <c r="AY3" s="60"/>
       <c r="AZ3" s="29"/>
       <c r="BA3" s="29"/>
-      <c r="BB3" s="56" t="s">
+      <c r="BB3" s="57" t="s">
         <v>213</v>
       </c>
-      <c r="BC3" s="57"/>
-      <c r="BD3" s="58"/>
+      <c r="BC3" s="58"/>
+      <c r="BD3" s="60"/>
       <c r="BE3" s="29"/>
       <c r="BF3" s="29"/>
-      <c r="BG3" s="56" t="s">
+      <c r="BG3" s="57" t="s">
         <v>214</v>
       </c>
-      <c r="BH3" s="57"/>
+      <c r="BH3" s="58"/>
       <c r="BI3" s="59"/>
       <c r="BJ3" s="31"/>
       <c r="BK3" s="32"/>

</xml_diff>